<commit_message>
finalisation calibration T2 - T1
</commit_message>
<xml_diff>
--- a/data/07_QUARTERLY_WEIGHTING/2024/T4/312X_1D/LFS_KNOWN_TOTALS_2024_T4_312X_1D.xlsx
+++ b/data/07_QUARTERLY_WEIGHTING/2024/T4/312X_1D/LFS_KNOWN_TOTALS_2024_T4_312X_1D.xlsx
@@ -2075,793 +2075,793 @@
         <v>980703</v>
       </c>
       <c r="AY2">
-        <v>2340645</v>
+        <v>0</v>
       </c>
       <c r="AZ2">
         <v>1035453</v>
       </c>
       <c r="BA2">
-        <v>2332825</v>
+        <v>0</v>
       </c>
       <c r="BB2">
         <v>153622</v>
       </c>
       <c r="BC2">
-        <v>257268</v>
+        <v>0</v>
       </c>
       <c r="BD2">
         <v>150819</v>
       </c>
       <c r="BE2">
-        <v>242739</v>
+        <v>0</v>
       </c>
       <c r="BF2">
         <v>112454</v>
       </c>
       <c r="BG2">
-        <v>188139</v>
+        <v>0</v>
       </c>
       <c r="BH2">
         <v>116539</v>
       </c>
       <c r="BI2">
-        <v>185974</v>
+        <v>0</v>
       </c>
       <c r="BJ2">
         <v>154331</v>
       </c>
       <c r="BK2">
-        <v>295872</v>
+        <v>0</v>
       </c>
       <c r="BL2">
         <v>154756</v>
       </c>
       <c r="BM2">
-        <v>281597</v>
+        <v>0</v>
       </c>
       <c r="BN2">
         <v>61378</v>
       </c>
       <c r="BO2">
-        <v>116835</v>
+        <v>0</v>
       </c>
       <c r="BP2">
         <v>61307</v>
       </c>
       <c r="BQ2">
-        <v>111296</v>
+        <v>0</v>
       </c>
       <c r="BR2">
         <v>108291</v>
       </c>
       <c r="BS2">
-        <v>172404</v>
+        <v>0</v>
       </c>
       <c r="BT2">
         <v>103529</v>
       </c>
       <c r="BU2">
-        <v>159424</v>
+        <v>0</v>
       </c>
       <c r="BV2">
         <v>48843</v>
       </c>
       <c r="BW2">
-        <v>105586</v>
+        <v>0</v>
       </c>
       <c r="BX2">
         <v>52389</v>
       </c>
       <c r="BY2">
-        <v>105152</v>
+        <v>0</v>
       </c>
       <c r="BZ2">
         <v>49603</v>
       </c>
       <c r="CA2">
-        <v>91882</v>
+        <v>0</v>
       </c>
       <c r="CB2">
         <v>49540</v>
       </c>
       <c r="CC2">
-        <v>91111</v>
+        <v>0</v>
       </c>
       <c r="CD2">
         <v>87456</v>
       </c>
       <c r="CE2">
-        <v>159390</v>
+        <v>0</v>
       </c>
       <c r="CF2">
         <v>88018</v>
       </c>
       <c r="CG2">
-        <v>142563</v>
+        <v>0</v>
       </c>
       <c r="CH2">
         <v>25076</v>
       </c>
       <c r="CI2">
-        <v>38606</v>
+        <v>0</v>
       </c>
       <c r="CJ2">
         <v>24122</v>
       </c>
       <c r="CK2">
-        <v>35405</v>
+        <v>0</v>
       </c>
       <c r="CL2">
         <v>15740</v>
       </c>
       <c r="CM2">
-        <v>28550</v>
+        <v>0</v>
       </c>
       <c r="CN2">
         <v>16241</v>
       </c>
       <c r="CO2">
-        <v>30118</v>
+        <v>0</v>
       </c>
       <c r="CP2">
         <v>88490</v>
       </c>
       <c r="CQ2">
-        <v>144074</v>
+        <v>0</v>
       </c>
       <c r="CR2">
         <v>84930</v>
       </c>
       <c r="CS2">
-        <v>134015</v>
+        <v>0</v>
       </c>
       <c r="CT2">
         <v>63228</v>
       </c>
       <c r="CU2">
-        <v>126637</v>
+        <v>0</v>
       </c>
       <c r="CV2">
         <v>63206</v>
       </c>
       <c r="CW2">
-        <v>126569</v>
+        <v>0</v>
       </c>
       <c r="CX2">
         <v>31343</v>
       </c>
       <c r="CY2">
-        <v>47443</v>
+        <v>0</v>
       </c>
       <c r="CZ2">
         <v>30962</v>
       </c>
       <c r="DA2">
-        <v>44075</v>
+        <v>0</v>
       </c>
       <c r="DB2">
         <v>94153</v>
       </c>
       <c r="DC2">
-        <v>157492</v>
+        <v>0</v>
       </c>
       <c r="DD2">
         <v>93692</v>
       </c>
       <c r="DE2">
-        <v>149860</v>
+        <v>0</v>
       </c>
       <c r="DF2">
         <v>74063</v>
       </c>
       <c r="DG2">
-        <v>137896</v>
+        <v>0</v>
       </c>
       <c r="DH2">
         <v>74064</v>
       </c>
       <c r="DI2">
-        <v>131465</v>
+        <v>0</v>
       </c>
       <c r="DJ2">
         <v>92544</v>
       </c>
       <c r="DK2">
-        <v>153003</v>
+        <v>0</v>
       </c>
       <c r="DL2">
         <v>92979</v>
       </c>
       <c r="DM2">
-        <v>148637</v>
+        <v>0</v>
       </c>
       <c r="DN2">
         <v>61966</v>
       </c>
       <c r="DO2">
-        <v>113220</v>
+        <v>0</v>
       </c>
       <c r="DP2">
         <v>60240</v>
       </c>
       <c r="DQ2">
-        <v>89828</v>
+        <v>0</v>
       </c>
       <c r="DR2">
         <v>13977</v>
       </c>
       <c r="DS2">
-        <v>20377</v>
+        <v>0</v>
       </c>
       <c r="DT2">
         <v>13531</v>
       </c>
       <c r="DU2">
-        <v>18754</v>
+        <v>0</v>
       </c>
       <c r="DV2">
         <v>51017</v>
       </c>
       <c r="DW2">
-        <v>74468</v>
+        <v>0</v>
       </c>
       <c r="DX2">
         <v>50958</v>
       </c>
       <c r="DY2">
-        <v>72391</v>
+        <v>0</v>
       </c>
       <c r="DZ2">
         <v>28759</v>
       </c>
       <c r="EA2">
-        <v>54131</v>
+        <v>0</v>
       </c>
       <c r="EB2">
         <v>28763</v>
       </c>
       <c r="EC2">
-        <v>51122</v>
+        <v>0</v>
       </c>
       <c r="ED2">
         <v>24860</v>
       </c>
       <c r="EE2">
-        <v>35860</v>
+        <v>0</v>
       </c>
       <c r="EF2">
         <v>23885</v>
       </c>
       <c r="EG2">
-        <v>33302</v>
+        <v>0</v>
       </c>
       <c r="EH2">
         <v>16737</v>
       </c>
       <c r="EI2">
-        <v>28266</v>
+        <v>0</v>
       </c>
       <c r="EJ2">
         <v>16595</v>
       </c>
       <c r="EK2">
-        <v>27349</v>
+        <v>0</v>
       </c>
       <c r="EL2">
         <v>7824</v>
       </c>
       <c r="EM2">
-        <v>10133</v>
+        <v>0</v>
       </c>
       <c r="EN2">
         <v>7452</v>
       </c>
       <c r="EO2">
-        <v>9606</v>
+        <v>0</v>
       </c>
       <c r="EP2">
         <v>25449</v>
       </c>
       <c r="EQ2">
-        <v>42784</v>
+        <v>0</v>
       </c>
       <c r="ER2">
         <v>24956</v>
       </c>
       <c r="ES2">
-        <v>35347</v>
+        <v>0</v>
       </c>
       <c r="ET2">
         <v>38160</v>
       </c>
       <c r="EU2">
-        <v>72633</v>
+        <v>0</v>
       </c>
       <c r="EV2">
         <v>38810</v>
       </c>
       <c r="EW2">
-        <v>70495</v>
+        <v>0</v>
       </c>
       <c r="EX2">
         <v>73041</v>
       </c>
       <c r="EY2">
-        <v>117794</v>
+        <v>0</v>
       </c>
       <c r="EZ2">
         <v>69075</v>
       </c>
       <c r="FA2">
-        <v>103510</v>
+        <v>0</v>
       </c>
       <c r="FB2">
         <v>49549</v>
       </c>
       <c r="FC2">
-        <v>85706</v>
+        <v>0</v>
       </c>
       <c r="FD2">
         <v>49694</v>
       </c>
       <c r="FE2">
-        <v>80849</v>
+        <v>0</v>
       </c>
       <c r="FF2">
         <v>24649</v>
       </c>
       <c r="FG2">
-        <v>44212</v>
+        <v>0</v>
       </c>
       <c r="FH2">
         <v>24435</v>
       </c>
       <c r="FI2">
-        <v>42090</v>
+        <v>0</v>
       </c>
       <c r="FJ2">
         <v>61362</v>
       </c>
       <c r="FK2">
-        <v>124511</v>
+        <v>0</v>
       </c>
       <c r="FL2">
         <v>59140</v>
       </c>
       <c r="FM2">
-        <v>118104</v>
+        <v>0</v>
       </c>
       <c r="FN2">
         <v>83778</v>
       </c>
       <c r="FO2">
-        <v>138133</v>
+        <v>0</v>
       </c>
       <c r="FP2">
         <v>81070</v>
       </c>
       <c r="FQ2">
-        <v>122465</v>
+        <v>0</v>
       </c>
       <c r="FR2">
         <v>49839</v>
       </c>
       <c r="FS2">
-        <v>78097</v>
+        <v>0</v>
       </c>
       <c r="FT2">
         <v>50104</v>
       </c>
       <c r="FU2">
-        <v>77001</v>
+        <v>0</v>
       </c>
       <c r="FV2">
         <v>32120</v>
       </c>
       <c r="FW2">
-        <v>62315</v>
+        <v>0</v>
       </c>
       <c r="FX2">
         <v>30629</v>
       </c>
       <c r="FY2">
-        <v>59344</v>
+        <v>0</v>
       </c>
       <c r="FZ2">
         <v>28606</v>
       </c>
       <c r="GA2">
-        <v>61850</v>
+        <v>0</v>
       </c>
       <c r="GB2">
         <v>28756</v>
       </c>
       <c r="GC2">
-        <v>56468</v>
+        <v>0</v>
       </c>
       <c r="GD2">
         <v>228138</v>
       </c>
       <c r="GE2">
-        <v>310186</v>
+        <v>0</v>
       </c>
       <c r="GF2">
         <v>210806</v>
       </c>
       <c r="GG2">
-        <v>282480</v>
+        <v>0</v>
       </c>
       <c r="GH2">
         <v>121106</v>
       </c>
       <c r="GI2">
-        <v>142752</v>
+        <v>0</v>
       </c>
       <c r="GJ2">
         <v>120156</v>
       </c>
       <c r="GK2">
-        <v>161860</v>
+        <v>0</v>
       </c>
       <c r="GL2">
         <v>117988</v>
       </c>
       <c r="GM2">
-        <v>153486</v>
+        <v>0</v>
       </c>
       <c r="GN2">
         <v>109396</v>
       </c>
       <c r="GO2">
-        <v>165485</v>
+        <v>0</v>
       </c>
       <c r="GP2">
         <v>87265</v>
       </c>
       <c r="GQ2">
-        <v>133953</v>
+        <v>0</v>
       </c>
       <c r="GR2">
         <v>81487</v>
       </c>
       <c r="GS2">
-        <v>113715</v>
+        <v>0</v>
       </c>
       <c r="GT2">
         <v>215925</v>
       </c>
       <c r="GU2">
-        <v>288337</v>
+        <v>0</v>
       </c>
       <c r="GV2">
         <v>198574</v>
       </c>
       <c r="GW2">
-        <v>258783</v>
+        <v>0</v>
       </c>
       <c r="GX2">
         <v>25814</v>
       </c>
       <c r="GY2">
-        <v>44660</v>
+        <v>0</v>
       </c>
       <c r="GZ2">
         <v>23751</v>
       </c>
       <c r="HA2">
-        <v>42021</v>
+        <v>0</v>
       </c>
       <c r="HB2">
         <v>145483</v>
       </c>
       <c r="HC2">
-        <v>204314</v>
+        <v>0</v>
       </c>
       <c r="HD2">
         <v>136439</v>
       </c>
       <c r="HE2">
-        <v>210415</v>
+        <v>0</v>
       </c>
       <c r="HF2">
         <v>137274</v>
       </c>
       <c r="HG2">
-        <v>218124</v>
+        <v>0</v>
       </c>
       <c r="HH2">
         <v>133732</v>
       </c>
       <c r="HI2">
-        <v>175911</v>
+        <v>0</v>
       </c>
       <c r="HJ2">
         <v>44150</v>
       </c>
       <c r="HK2">
-        <v>50464</v>
+        <v>0</v>
       </c>
       <c r="HL2">
         <v>41305</v>
       </c>
       <c r="HM2">
-        <v>51848</v>
+        <v>0</v>
       </c>
       <c r="HN2">
         <v>36778</v>
       </c>
       <c r="HO2">
-        <v>50444</v>
+        <v>0</v>
       </c>
       <c r="HP2">
         <v>34798</v>
       </c>
       <c r="HQ2">
-        <v>54255</v>
+        <v>0</v>
       </c>
       <c r="HR2">
         <v>130557</v>
       </c>
       <c r="HS2">
-        <v>180384</v>
+        <v>0</v>
       </c>
       <c r="HT2">
         <v>120597</v>
       </c>
       <c r="HU2">
-        <v>164153</v>
+        <v>0</v>
       </c>
       <c r="HV2">
         <v>87421</v>
       </c>
       <c r="HW2">
-        <v>146391</v>
+        <v>0</v>
       </c>
       <c r="HX2">
         <v>85658</v>
       </c>
       <c r="HY2">
-        <v>134813</v>
+        <v>0</v>
       </c>
       <c r="HZ2">
         <v>75703</v>
       </c>
       <c r="IA2">
-        <v>91567</v>
+        <v>0</v>
       </c>
       <c r="IB2">
         <v>72072</v>
       </c>
       <c r="IC2">
-        <v>86596</v>
+        <v>0</v>
       </c>
       <c r="ID2">
         <v>146755</v>
       </c>
       <c r="IE2">
-        <v>207603</v>
+        <v>0</v>
       </c>
       <c r="IF2">
         <v>142211</v>
       </c>
       <c r="IG2">
-        <v>191974</v>
+        <v>0</v>
       </c>
       <c r="IH2">
         <v>98438</v>
       </c>
       <c r="II2">
-        <v>169435</v>
+        <v>0</v>
       </c>
       <c r="IJ2">
         <v>94635</v>
       </c>
       <c r="IK2">
-        <v>147014</v>
+        <v>0</v>
       </c>
       <c r="IL2">
         <v>122597</v>
       </c>
       <c r="IM2">
-        <v>171530</v>
+        <v>0</v>
       </c>
       <c r="IN2">
         <v>117368</v>
       </c>
       <c r="IO2">
-        <v>156449</v>
+        <v>0</v>
       </c>
       <c r="IP2">
         <v>96070</v>
       </c>
       <c r="IQ2">
-        <v>155271</v>
+        <v>0</v>
       </c>
       <c r="IR2">
         <v>86757</v>
       </c>
       <c r="IS2">
-        <v>117993</v>
+        <v>0</v>
       </c>
       <c r="IT2">
         <v>48602</v>
       </c>
       <c r="IU2">
-        <v>60977</v>
+        <v>0</v>
       </c>
       <c r="IV2">
         <v>46360</v>
       </c>
       <c r="IW2">
-        <v>60353</v>
+        <v>0</v>
       </c>
       <c r="IX2">
         <v>72444</v>
       </c>
       <c r="IY2">
-        <v>87264</v>
+        <v>0</v>
       </c>
       <c r="IZ2">
         <v>69650</v>
       </c>
       <c r="JA2">
-        <v>90700</v>
+        <v>0</v>
       </c>
       <c r="JB2">
         <v>59378</v>
       </c>
       <c r="JC2">
-        <v>79946</v>
+        <v>0</v>
       </c>
       <c r="JD2">
         <v>56540</v>
       </c>
       <c r="JE2">
-        <v>86618</v>
+        <v>0</v>
       </c>
       <c r="JF2">
         <v>100227</v>
       </c>
       <c r="JG2">
-        <v>117002</v>
+        <v>0</v>
       </c>
       <c r="JH2">
         <v>94208</v>
       </c>
       <c r="JI2">
-        <v>116902</v>
+        <v>0</v>
       </c>
       <c r="JJ2">
         <v>91181</v>
       </c>
       <c r="JK2">
-        <v>98330</v>
+        <v>0</v>
       </c>
       <c r="JL2">
         <v>88479</v>
       </c>
       <c r="JM2">
-        <v>107062</v>
+        <v>0</v>
       </c>
       <c r="JN2">
         <v>30503</v>
       </c>
       <c r="JO2">
-        <v>32936</v>
+        <v>0</v>
       </c>
       <c r="JP2">
         <v>29112</v>
       </c>
       <c r="JQ2">
-        <v>33387</v>
+        <v>0</v>
       </c>
       <c r="JR2">
         <v>79315</v>
       </c>
       <c r="JS2">
-        <v>117644</v>
+        <v>0</v>
       </c>
       <c r="JT2">
         <v>74829</v>
       </c>
       <c r="JU2">
-        <v>98039</v>
+        <v>0</v>
       </c>
       <c r="JV2">
         <v>50230</v>
       </c>
       <c r="JW2">
-        <v>81886</v>
+        <v>0</v>
       </c>
       <c r="JX2">
         <v>48085</v>
       </c>
       <c r="JY2">
-        <v>74540</v>
+        <v>0</v>
       </c>
       <c r="JZ2">
         <v>139994</v>
       </c>
       <c r="KA2">
-        <v>207789</v>
+        <v>0</v>
       </c>
       <c r="KB2">
         <v>128293</v>
       </c>
       <c r="KC2">
-        <v>177314</v>
+        <v>0</v>
       </c>
       <c r="KD2">
         <v>85630</v>
       </c>
       <c r="KE2">
-        <v>125144</v>
+        <v>0</v>
       </c>
       <c r="KF2">
         <v>81554</v>
       </c>
       <c r="KG2">
-        <v>116827</v>
+        <v>0</v>
       </c>
       <c r="KH2">
         <v>56827</v>
       </c>
       <c r="KI2">
-        <v>77479</v>
+        <v>0</v>
       </c>
       <c r="KJ2">
         <v>52973</v>
       </c>
       <c r="KK2">
-        <v>79665</v>
+        <v>0</v>
       </c>
       <c r="KL2">
         <v>74817</v>
       </c>
       <c r="KM2">
-        <v>142403</v>
+        <v>0</v>
       </c>
       <c r="KN2">
         <v>70630</v>
       </c>
       <c r="KO2">
-        <v>133468</v>
+        <v>0</v>
       </c>
       <c r="KP2">
         <v>174209</v>
       </c>
       <c r="KQ2">
-        <v>249144</v>
+        <v>0</v>
       </c>
       <c r="KR2">
         <v>169615</v>
       </c>
       <c r="KS2">
-        <v>219637</v>
+        <v>0</v>
       </c>
       <c r="KT2">
         <v>97870</v>
       </c>
       <c r="KU2">
-        <v>109521</v>
+        <v>0</v>
       </c>
       <c r="KV2">
         <v>93707</v>
       </c>
       <c r="KW2">
-        <v>114264</v>
+        <v>0</v>
       </c>
       <c r="KX2">
         <v>51625</v>
       </c>
       <c r="KY2">
-        <v>100926</v>
+        <v>0</v>
       </c>
       <c r="KZ2">
         <v>46521</v>
       </c>
       <c r="LA2">
-        <v>86117</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>